<commit_message>
Corrida | SFE-CEM | 2026-06-12 10:37:08.995846
</commit_message>
<xml_diff>
--- a/indicadores/SFE-CEM_out.xlsx
+++ b/indicadores/SFE-CEM_out.xlsx
@@ -22719,237 +22719,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B999F33F-7FB0-4E6D-A1CC-F1F0B93197B4}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8809E3E5-B463-4607-A23E-CCA491129191}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBF039C2-840B-47A1-8E9F-CFED83804BDF}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | SFE-CEM | 2026-06-22 11:40:45.02494
</commit_message>
<xml_diff>
--- a/indicadores/SFE-CEM_out.xlsx
+++ b/indicadores/SFE-CEM_out.xlsx
@@ -113,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">17/06/2026</t>
+    <t xml:space="preserve">22/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">focampo</t>
+    <t xml:space="preserve">arodriguez</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1930,9 +1930,7 @@
       <c r="J7" s="1"/>
     </row>
     <row r="8">
-      <c r="A8" t="s">
-        <v>21</v>
-      </c>
+      <c r="A8"/>
       <c r="B8"/>
       <c r="C8"/>
       <c r="D8"/>
@@ -1944,14 +1942,10 @@
       <c r="J8" s="1"/>
     </row>
     <row r="9">
-      <c r="A9" t="s">
-        <v>22</v>
-      </c>
+      <c r="A9"/>
       <c r="B9"/>
       <c r="C9"/>
-      <c r="D9" t="n">
-        <v>0.601644398112104</v>
-      </c>
+      <c r="D9"/>
       <c r="E9"/>
       <c r="F9"/>
       <c r="G9"/>
@@ -1961,13 +1955,11 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
-      <c r="D10" t="n">
-        <v>0</v>
-      </c>
+      <c r="D10"/>
       <c r="E10"/>
       <c r="F10"/>
       <c r="G10"/>
@@ -1976,10 +1968,14 @@
       <c r="J10" s="1"/>
     </row>
     <row r="11">
-      <c r="A11"/>
+      <c r="A11" t="s">
+        <v>22</v>
+      </c>
       <c r="B11"/>
       <c r="C11"/>
-      <c r="D11"/>
+      <c r="D11" t="n">
+        <v>0.621769881888537</v>
+      </c>
       <c r="E11"/>
       <c r="F11"/>
       <c r="G11"/>
@@ -1989,11 +1985,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
-      <c r="D12"/>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
       <c r="E12"/>
       <c r="F12"/>
       <c r="G12"/>
@@ -2002,14 +2000,10 @@
       <c r="J12" s="1"/>
     </row>
     <row r="13">
-      <c r="A13" t="s">
-        <v>25</v>
-      </c>
+      <c r="A13"/>
       <c r="B13"/>
       <c r="C13"/>
-      <c r="D13" t="n">
-        <v>0.361975981779676</v>
-      </c>
+      <c r="D13"/>
       <c r="E13"/>
       <c r="F13"/>
       <c r="G13"/>
@@ -2018,7 +2012,9 @@
       <c r="J13" s="1"/>
     </row>
     <row r="14">
-      <c r="A14"/>
+      <c r="A14" t="s">
+        <v>24</v>
+      </c>
       <c r="B14"/>
       <c r="C14"/>
       <c r="D14"/>
@@ -2031,11 +2027,13 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
-      <c r="D15"/>
+      <c r="D15" t="n">
+        <v>0.386597786023685</v>
+      </c>
       <c r="E15"/>
       <c r="F15"/>
       <c r="G15"/>
@@ -2044,9 +2042,7 @@
       <c r="J15" s="1"/>
     </row>
     <row r="16">
-      <c r="A16" t="s">
-        <v>27</v>
-      </c>
+      <c r="A16"/>
       <c r="B16"/>
       <c r="C16"/>
       <c r="D16"/>
@@ -2059,7 +2055,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2073,13 +2069,11 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
-      <c r="D18" t="n">
-        <v>0.00193629710151174</v>
-      </c>
+      <c r="D18"/>
       <c r="E18"/>
       <c r="F18"/>
       <c r="G18"/>
@@ -2089,7 +2083,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2108,7 +2102,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.0629759188996908</v>
+        <v>0.00212288808246272</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2118,7 +2112,9 @@
       <c r="J20" s="1"/>
     </row>
     <row r="21">
-      <c r="A21"/>
+      <c r="A21" t="s">
+        <v>30</v>
+      </c>
       <c r="B21"/>
       <c r="C21"/>
       <c r="D21"/>
@@ -2130,10 +2126,14 @@
       <c r="J21" s="1"/>
     </row>
     <row r="22">
-      <c r="A22"/>
+      <c r="A22" t="s">
+        <v>29</v>
+      </c>
       <c r="B22"/>
       <c r="C22"/>
-      <c r="D22"/>
+      <c r="D22" t="n">
+        <v>0.0365094510809262</v>
+      </c>
       <c r="E22"/>
       <c r="F22"/>
       <c r="G22"/>
@@ -22557,7 +22557,7 @@
         <v>447</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.0683133946393464</v>
+        <v>0.0666904593246495</v>
       </c>
     </row>
     <row r="6">
@@ -22565,7 +22565,7 @@
         <v>448</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.119731826752879</v>
+        <v>0.11766684980448</v>
       </c>
     </row>
     <row r="7">
@@ -22573,7 +22573,7 @@
         <v>449</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.182263728812132</v>
+        <v>0.180298929560288</v>
       </c>
     </row>
     <row r="8">
@@ -22581,7 +22581,7 @@
         <v>450</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.281184219594645</v>
+        <v>0.280818065603805</v>
       </c>
     </row>
     <row r="9">
@@ -22589,7 +22589,7 @@
         <v>451</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.38169875729018</v>
+        <v>0.376270806192053</v>
       </c>
     </row>
     <row r="10">
@@ -22597,7 +22597,7 @@
         <v>452</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.434781900756177</v>
+        <v>0.427392334528196</v>
       </c>
     </row>
     <row r="11">
@@ -22605,7 +22605,7 @@
         <v>453</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.469197800289005</v>
+        <v>0.468024038336903</v>
       </c>
     </row>
     <row r="12">
@@ -22613,7 +22613,7 @@
         <v>454</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.496566909349702</v>
+        <v>0.50132866832126</v>
       </c>
     </row>
     <row r="13">
@@ -22621,7 +22621,7 @@
         <v>455</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.562131095578262</v>
+        <v>0.575686423223806</v>
       </c>
     </row>
     <row r="14">
@@ -22629,7 +22629,7 @@
         <v>456</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.601644398112104</v>
+        <v>0.621769881888537</v>
       </c>
     </row>
     <row r="15">
@@ -22637,7 +22637,7 @@
         <v>457</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.487668679978274</v>
+        <v>0.503235758940932</v>
       </c>
     </row>
     <row r="16">
@@ -22645,7 +22645,7 @@
         <v>458</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.334736698910662</v>
+        <v>0.343277295538825</v>
       </c>
     </row>
     <row r="17">
@@ -22653,7 +22653,7 @@
         <v>459</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.232512488370671</v>
+        <v>0.239215206751941</v>
       </c>
     </row>
     <row r="18">
@@ -22661,7 +22661,7 @@
         <v>460</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.157433480278266</v>
+        <v>0.163384952787316</v>
       </c>
     </row>
     <row r="19">
@@ -22669,7 +22669,7 @@
         <v>461</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.0994762932188359</v>
+        <v>0.0994319963585631</v>
       </c>
     </row>
     <row r="20">
@@ -22677,7 +22677,7 @@
         <v>462</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.00770141193522336</v>
+        <v>0.00362842220210238</v>
       </c>
     </row>
     <row r="21">
@@ -22685,7 +22685,7 @@
         <v>463</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.0740681115564446</v>
+        <v>-0.075085637827108</v>
       </c>
     </row>
     <row r="22">
@@ -22693,7 +22693,7 @@
         <v>464</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.107037584289077</v>
+        <v>-0.104081856013497</v>
       </c>
     </row>
     <row r="23">
@@ -22701,7 +22701,7 @@
         <v>465</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.122986426762152</v>
+        <v>-0.119384224581923</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-CEM | 2026-07-15 08:38:30.292542
</commit_message>
<xml_diff>
--- a/indicadores/SFE-CEM_out.xlsx
+++ b/indicadores/SFE-CEM_out.xlsx
@@ -113,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">13/07/2026</t>
+    <t xml:space="preserve">15/07/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">ysonder</t>
+    <t xml:space="preserve">pcohan</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1974,7 +1974,7 @@
       <c r="B11"/>
       <c r="C11"/>
       <c r="D11" t="n">
-        <v>0.622073798389017</v>
+        <v>0.623753602101325</v>
       </c>
       <c r="E11"/>
       <c r="F11"/>
@@ -2032,7 +2032,7 @@
       <c r="B15"/>
       <c r="C15"/>
       <c r="D15" t="n">
-        <v>0.386975810642139</v>
+        <v>0.389068556134377</v>
       </c>
       <c r="E15"/>
       <c r="F15"/>
@@ -2102,7 +2102,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.00354503426569496</v>
+        <v>0.00292098337288874</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2132,7 +2132,7 @@
       <c r="B22"/>
       <c r="C22"/>
       <c r="D22" t="n">
-        <v>0.00308801537895245</v>
+        <v>0.00324486561350824</v>
       </c>
       <c r="E22"/>
       <c r="F22"/>
@@ -22593,7 +22593,7 @@
         <v>447</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.0730883398981323</v>
+        <v>0.074391572556599</v>
       </c>
     </row>
     <row r="6">
@@ -22601,7 +22601,7 @@
         <v>448</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.12038349708555</v>
+        <v>0.121612003949296</v>
       </c>
     </row>
     <row r="7">
@@ -22609,7 +22609,7 @@
         <v>449</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.18103231401009</v>
+        <v>0.178424051166914</v>
       </c>
     </row>
     <row r="8">
@@ -22617,7 +22617,7 @@
         <v>450</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.286663877445563</v>
+        <v>0.282620043619112</v>
       </c>
     </row>
     <row r="9">
@@ -22625,7 +22625,7 @@
         <v>451</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.385052184492687</v>
+        <v>0.384846231209228</v>
       </c>
     </row>
     <row r="10">
@@ -22633,7 +22633,7 @@
         <v>452</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.434148319663633</v>
+        <v>0.434095476970319</v>
       </c>
     </row>
     <row r="11">
@@ -22641,7 +22641,7 @@
         <v>453</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.472555499980118</v>
+        <v>0.470745241016989</v>
       </c>
     </row>
     <row r="12">
@@ -22649,7 +22649,7 @@
         <v>454</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.504469646764607</v>
+        <v>0.50348412347554</v>
       </c>
     </row>
     <row r="13">
@@ -22657,7 +22657,7 @@
         <v>455</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.576253592451772</v>
+        <v>0.575812903925237</v>
       </c>
     </row>
     <row r="14">
@@ -22665,7 +22665,7 @@
         <v>456</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.622073798389017</v>
+        <v>0.623753602101325</v>
       </c>
     </row>
     <row r="15">
@@ -22673,7 +22673,7 @@
         <v>457</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.509933516260939</v>
+        <v>0.510983487382165</v>
       </c>
     </row>
     <row r="16">
@@ -22681,7 +22681,7 @@
         <v>458</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.349299794681194</v>
+        <v>0.347256560182168</v>
       </c>
     </row>
     <row r="17">
@@ -22689,7 +22689,7 @@
         <v>459</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.242890749873187</v>
+        <v>0.241417493749056</v>
       </c>
     </row>
     <row r="18">
@@ -22697,7 +22697,7 @@
         <v>460</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.164063726133365</v>
+        <v>0.162037016881693</v>
       </c>
     </row>
     <row r="19">
@@ -22705,7 +22705,7 @@
         <v>461</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.0955467914851817</v>
+        <v>0.090989298401641</v>
       </c>
     </row>
     <row r="20">
@@ -22713,7 +22713,7 @@
         <v>462</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.00137457999239488</v>
+        <v>0.000141237978774124</v>
       </c>
     </row>
     <row r="21">
@@ -22721,7 +22721,7 @@
         <v>463</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.071993204097546</v>
+        <v>-0.0708119201432514</v>
       </c>
     </row>
     <row r="22">
@@ -22729,7 +22729,7 @@
         <v>464</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.101206391425949</v>
+        <v>-0.101451149258678</v>
       </c>
     </row>
     <row r="23">
@@ -22737,7 +22737,7 @@
         <v>465</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.121251187263589</v>
+        <v>-0.120465692353494</v>
       </c>
     </row>
     <row r="24">
@@ -22765,237 +22765,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D84A982-C9FB-451A-80CE-47CCFD310F0A}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C02E2D40-2245-4D9A-AABF-0C35EBBBF188}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4711A300-6886-437A-96C9-6DD0A6CCBE34}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | SFE-CEM | 2026-08-27 11:08:32.10665
</commit_message>
<xml_diff>
--- a/indicadores/SFE-CEM_out.xlsx
+++ b/indicadores/SFE-CEM_out.xlsx
@@ -1974,7 +1974,7 @@
       <c r="B11"/>
       <c r="C11"/>
       <c r="D11" t="n">
-        <v>0.583047364511345</v>
+        <v>0.586184693535749</v>
       </c>
       <c r="E11"/>
       <c r="F11"/>
@@ -2032,7 +2032,7 @@
       <c r="B15"/>
       <c r="C15"/>
       <c r="D15" t="n">
-        <v>0.339944229263625</v>
+        <v>0.3436124949356</v>
       </c>
       <c r="E15"/>
       <c r="F15"/>
@@ -2102,7 +2102,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.0174171232341642</v>
+        <v>0.014917436833102</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2132,7 +2132,7 @@
       <c r="B22"/>
       <c r="C22"/>
       <c r="D22" t="n">
-        <v>0.0287831394923482</v>
+        <v>0.0389530266315721</v>
       </c>
       <c r="E22"/>
       <c r="F22"/>
@@ -22629,7 +22629,7 @@
         <v>447</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.0361510506971771</v>
+        <v>0.0338700660339597</v>
       </c>
     </row>
     <row r="6">
@@ -22637,7 +22637,7 @@
         <v>448</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.105547929004201</v>
+        <v>0.106738384220886</v>
       </c>
     </row>
     <row r="7">
@@ -22645,7 +22645,7 @@
         <v>449</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.180814829624127</v>
+        <v>0.184561674929964</v>
       </c>
     </row>
     <row r="8">
@@ -22653,7 +22653,7 @@
         <v>450</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.268218535467819</v>
+        <v>0.270204488872229</v>
       </c>
     </row>
     <row r="9">
@@ -22661,7 +22661,7 @@
         <v>451</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.36720382202138</v>
+        <v>0.364896781556905</v>
       </c>
     </row>
     <row r="10">
@@ -22669,7 +22669,7 @@
         <v>452</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.421053052885453</v>
+        <v>0.413637168119874</v>
       </c>
     </row>
     <row r="11">
@@ -22677,7 +22677,7 @@
         <v>453</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.431659241025372</v>
+        <v>0.42234493952333</v>
       </c>
     </row>
     <row r="12">
@@ -22685,7 +22685,7 @@
         <v>454</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.452237555899594</v>
+        <v>0.447019379355878</v>
       </c>
     </row>
     <row r="13">
@@ -22693,7 +22693,7 @@
         <v>455</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.535075708231134</v>
+        <v>0.535208950471958</v>
       </c>
     </row>
     <row r="14">
@@ -22701,7 +22701,7 @@
         <v>456</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.583047364511345</v>
+        <v>0.586184693535749</v>
       </c>
     </row>
     <row r="15">
@@ -22709,7 +22709,7 @@
         <v>457</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.470014738278765</v>
+        <v>0.473758921153878</v>
       </c>
     </row>
     <row r="16">
@@ -22717,7 +22717,7 @@
         <v>458</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.311098416606633</v>
+        <v>0.314675954804637</v>
       </c>
     </row>
     <row r="17">
@@ -22725,7 +22725,7 @@
         <v>459</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.221351279412801</v>
+        <v>0.224229749682697</v>
       </c>
     </row>
     <row r="18">
@@ -22733,7 +22733,7 @@
         <v>460</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.16797253938449</v>
+        <v>0.167907760942385</v>
       </c>
     </row>
     <row r="19">
@@ -22741,7 +22741,7 @@
         <v>461</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.111879593555942</v>
+        <v>0.110562552406788</v>
       </c>
     </row>
     <row r="20">
@@ -22749,7 +22749,7 @@
         <v>462</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.0259910235595353</v>
+        <v>0.0268667261604762</v>
       </c>
     </row>
     <row r="21">
@@ -22757,7 +22757,7 @@
         <v>463</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.0464781345282008</v>
+        <v>-0.0438570674988556</v>
       </c>
     </row>
     <row r="22">
@@ -22765,7 +22765,7 @@
         <v>464</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.0756498279049735</v>
+        <v>-0.0720127021452785</v>
       </c>
     </row>
     <row r="23">
@@ -22773,7 +22773,7 @@
         <v>465</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.0762110009426667</v>
+        <v>-0.0738440617034069</v>
       </c>
     </row>
     <row r="24">

</xml_diff>